<commit_message>
95mm²-Offerte: 30% Marge verdeckt in die Einzelpreise einrechnen
Kalkulationsaufschlag von 30% wird auf jeden Artikelpreis aufgeschlagen
(Positions- und Artikelliste), statt als separate Zeile ausgewiesen.
Endbetrag steigt von 11'146.50 auf 14'490.45 CHF.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014S9DaLfa6MkaKKTKAHq7pF
</commit_message>
<xml_diff>
--- a/offerten/Offerte_Kabel_95mm.xlsx
+++ b/offerten/Offerte_Kabel_95mm.xlsx
@@ -856,7 +856,7 @@
         </is>
       </c>
       <c r="E22" s="18" t="n">
-        <v>234.2</v>
+        <v>304.46</v>
       </c>
       <c r="F22" s="16" t="n">
         <v>1</v>
@@ -889,7 +889,7 @@
         </is>
       </c>
       <c r="E23" s="22" t="n">
-        <v>2138.7</v>
+        <v>2780.31</v>
       </c>
       <c r="F23" s="20" t="n">
         <v>1</v>
@@ -922,7 +922,7 @@
         </is>
       </c>
       <c r="E24" s="18" t="n">
-        <v>160</v>
+        <v>208</v>
       </c>
       <c r="F24" s="16" t="n">
         <v>1</v>
@@ -1541,7 +1541,7 @@
         </is>
       </c>
       <c r="C2" s="38" t="n">
-        <v>234.2</v>
+        <v>304.46</v>
       </c>
     </row>
     <row r="3">
@@ -1556,7 +1556,7 @@
         </is>
       </c>
       <c r="C3" s="38" t="n">
-        <v>2138.7</v>
+        <v>2780.31</v>
       </c>
     </row>
     <row r="4">
@@ -1571,7 +1571,7 @@
         </is>
       </c>
       <c r="C4" s="38" t="n">
-        <v>2811.27</v>
+        <v>3654.65</v>
       </c>
     </row>
     <row r="5">
@@ -1586,7 +1586,7 @@
         </is>
       </c>
       <c r="C5" s="38" t="n">
-        <v>160</v>
+        <v>208</v>
       </c>
     </row>
   </sheetData>

</xml_diff>